<commit_message>
Excel: shapes in their outlines (Office's presets with their adjustments, LibreOffice's kinds and paths) and the theme's look as Excel's default shape (accent fill, darker outline, white words in the middle), from .xlsx and .ods; a combo's second value axis (a line on its own scale, its numbers at the right). shapes.py's and charts.py's workbooks, their .ods by LibreOffice; checked on the phone
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/src/test/resources/charts.xlsx
+++ b/app/src/test/resources/charts.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Combo" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Radar" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Bubble" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Two axes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -442,6 +443,132 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Sales and margin</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Two axes'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Two axes'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Two axes'!$B$2:$B$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Two axes'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Two axes'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="200"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="200"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crosses val="max"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -497,6 +624,33 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1074,4 +1228,88 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>